<commit_message>
Show pictures and charts in .xls and .ods workbooks
Excel 97-2003: pictures from the drawing group's picture store placed by their shape anchors; charts from their saved cache or from the saved cells their series refer to, including chart sheets. Sheet records after an embedded chart are no longer dropped. OpenDocument: pictures and chart objects anchored to cells or to the sheet, charts from their saved data table. Linked pictures are never opened. New fixtures and tests.
</commit_message>
<xml_diff>
--- a/tests/corpus/xlsx/attack-linked-picture.xlsx
+++ b/tests/corpus/xlsx/attack-linked-picture.xlsx
@@ -215,7 +215,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sales!$B$2:$B$5</c:f>
+              <c:f>Sales!$C$2:$C$5</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
@@ -304,7 +304,7 @@
           </c:tx>
           <c:cat>
             <c:strRef>
-              <c:f>Sales!$A$2:$A$5</c:f>
+              <c:f>Sales!$B$1:$C$1</c:f>
               <c:strCache>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
@@ -318,7 +318,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sales!$B$2:$B$5</c:f>
+              <c:f>Sales!$B$2:$C$2</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
@@ -463,7 +463,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sales!$B$2:$B$5</c:f>
+              <c:f>Sales!$C$2:$C$5</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>

</xml_diff>

<commit_message>
Show chart axis titles and data labels
Values in their number format, pie percentages and category names, read from .xlsx, .xls and .ods charts and drawn on the chart.
</commit_message>
<xml_diff>
--- a/tests/corpus/xlsx/attack-linked-picture.xlsx
+++ b/tests/corpus/xlsx/attack-linked-picture.xlsx
@@ -235,6 +235,14 @@
             </c:numRef>
           </c:val>
         </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
         <c:axId val="1"/>
         <c:axId val="2"/>
       </c:barChart>
@@ -245,6 +253,19 @@
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:r>
+                  <a:t>Month</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
         <c:crossAx val="2"/>
       </c:catAx>
       <c:valAx>
@@ -255,6 +276,19 @@
         <c:delete val="0"/>
         <c:axPos val="l"/>
         <c:majorGridlines/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:r>
+                  <a:t>Units sold</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
         <c:crossAx val="1"/>
       </c:valAx>
     </c:plotArea>
@@ -332,6 +366,14 @@
             </c:numRef>
           </c:val>
         </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="1"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="1"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
         <c:firstSliceAng val="0"/>
       </c:pieChart>
     </c:plotArea>

</xml_diff>